<commit_message>
Final Q3 submission package and audit for ETCCDI Chiang Mai project
Co-authored-by: surasit3173 <247266065+surasit3173@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ETCCDI_ChiangMai/audit/FIGURE_AUDIT.xlsx
+++ b/ETCCDI_ChiangMai/audit/FIGURE_AUDIT.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Figure_QA" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Figure_Audit" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -434,30 +434,25 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>No_Title_Inside_Artwork</t>
+          <t>Panel_Labels_Valid</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Panel_Labels_Valid</t>
+          <t>No_Overlap_Clipping</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>No_Overlap_Clipping</t>
+          <t>Correct_Units</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Correct_Units</t>
+          <t>Matches_Statistical_Tables</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
-        <is>
-          <t>Matches_Statistical_Tables</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
         <is>
           <t>QA_Status</t>
         </is>
@@ -471,11 +466,11 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2982x1179</t>
+          <t>3000x1200</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>299.9994</v>
+        <v>300</v>
       </c>
       <c r="D2" t="b">
         <v>1</v>
@@ -489,10 +484,7 @@
       <c r="G2" t="b">
         <v>1</v>
       </c>
-      <c r="H2" t="b">
-        <v>1</v>
-      </c>
-      <c r="I2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -506,11 +498,11 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2978x2383</t>
+          <t>3000x2400</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>299.9994</v>
+        <v>300</v>
       </c>
       <c r="D3" t="b">
         <v>1</v>
@@ -524,10 +516,7 @@
       <c r="G3" t="b">
         <v>1</v>
       </c>
-      <c r="H3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -541,11 +530,11 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2984x2383</t>
+          <t>3000x2400</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>299.9994</v>
+        <v>300</v>
       </c>
       <c r="D4" t="b">
         <v>1</v>
@@ -559,10 +548,7 @@
       <c r="G4" t="b">
         <v>1</v>
       </c>
-      <c r="H4" t="b">
-        <v>1</v>
-      </c>
-      <c r="I4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -576,11 +562,11 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2380x1480</t>
+          <t>3300x1350</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>299.9994</v>
+        <v>300</v>
       </c>
       <c r="D5" t="b">
         <v>1</v>
@@ -594,10 +580,7 @@
       <c r="G5" t="b">
         <v>1</v>
       </c>
-      <c r="H5" t="b">
-        <v>1</v>
-      </c>
-      <c r="I5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -611,11 +594,11 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2686x1780</t>
+          <t>3000x2100</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>299.9994</v>
+        <v>300</v>
       </c>
       <c r="D6" t="b">
         <v>1</v>
@@ -629,10 +612,7 @@
       <c r="G6" t="b">
         <v>1</v>
       </c>
-      <c r="H6" t="b">
-        <v>1</v>
-      </c>
-      <c r="I6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>

</xml_diff>